<commit_message>
Using calculated suction_location columns
</commit_message>
<xml_diff>
--- a/CL & CD Graphs of Injection & Suction.xlsx
+++ b/CL & CD Graphs of Injection & Suction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\casus\OneDrive\Desktop\AERO ORGANISED\MY WORK, PROJECTS ETC\RESEARCH &amp; PATENTS\ANUP SIR\Optimising_conference_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3BB6A7-753E-4FCC-9FE1-992D9B94FDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191C750A-457F-4825-AD64-D9D8BED37E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
   <si>
     <t>AOA</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>optimisation + stabilisation</t>
+  </si>
+  <si>
+    <t>Calculated_suction</t>
   </si>
 </sst>
 </file>
@@ -256,6 +259,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -265,7 +269,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2125,6 +2128,237 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-BA19-49B0-8FBC-D5E84C509E1F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'PICET 2025'!$AA$34</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Calculated_suction</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'PICET 2025'!$Y$36:$Y$63</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'PICET 2025'!$Z$36:$Z$63</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>1.16369025971786</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.24913354186229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.3442212751009299</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.43651239789754</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.5291609066156</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.63174028144106</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.73326314317009</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.8344830952098099</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.93633394708781</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.0452641518224799</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.1523191707020302</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2580761461679302</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.3777388265627799</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.49639794926521</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.6158093888716598</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.71094462300836</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.8522603082045999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.9719790976206601</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.0902094245203799</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3.2060834969884802</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.2979787911071998</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.3601181784771201</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>3.4029657145452501</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3.4253480456309799</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>3.44238874354058</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>3.4657011033449399</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>3.4827335625295399</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>3.49976602171414</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5EDF-499C-B978-F313F33FC22C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3429,7 +3663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AF35"/>
+  <dimension ref="B1:AF63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="20" max="20" width="23.140625" customWidth="1"/>
@@ -3437,29 +3671,30 @@
     <col min="22" max="22" width="19.28515625" customWidth="1"/>
     <col min="23" max="23" width="22.5703125" customWidth="1"/>
     <col min="24" max="24" width="18.85546875" customWidth="1"/>
+    <col min="27" max="27" width="12.5703125" customWidth="1"/>
     <col min="29" max="29" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:32" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="16"/>
-      <c r="G2" s="14" t="s">
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="17"/>
+      <c r="G2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="L2" s="14" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="L2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="17"/>
       <c r="R2" s="10"/>
       <c r="S2" s="10"/>
       <c r="T2" s="10"/>
@@ -3470,7 +3705,7 @@
       <c r="AB2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="17"/>
+      <c r="AC2" s="14"/>
       <c r="AD2" s="11"/>
     </row>
     <row r="4" spans="2:32" ht="15.75" x14ac:dyDescent="0.25">
@@ -5083,10 +5318,594 @@
         <v>600</v>
       </c>
     </row>
-    <row r="34" spans="21:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="21:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="21:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="21:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AA34" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB34" s="11"/>
+    </row>
+    <row r="35" spans="21:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="U35" s="13" t="s">
         <v>13</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z35" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y36">
+        <v>0</v>
+      </c>
+      <c r="Z36">
+        <v>1.16369025971786</v>
+      </c>
+      <c r="AA36">
+        <v>370</v>
+      </c>
+      <c r="AB36">
+        <v>1.4030768497089401</v>
+      </c>
+      <c r="AC36">
+        <v>2000000</v>
+      </c>
+      <c r="AD36">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="37" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y37">
+        <v>1</v>
+      </c>
+      <c r="Z37">
+        <v>1.24913354186229</v>
+      </c>
+      <c r="AA37">
+        <v>240</v>
+      </c>
+      <c r="AB37">
+        <v>0.81860430505974402</v>
+      </c>
+      <c r="AC37">
+        <v>2000000</v>
+      </c>
+      <c r="AD37">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="38" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y38">
+        <v>2</v>
+      </c>
+      <c r="Z38">
+        <v>1.3442212751009299</v>
+      </c>
+      <c r="AA38">
+        <v>240</v>
+      </c>
+      <c r="AB38">
+        <v>0.79606329054005198</v>
+      </c>
+      <c r="AC38">
+        <v>2000000</v>
+      </c>
+      <c r="AD38">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="39" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y39">
+        <v>3</v>
+      </c>
+      <c r="Z39">
+        <v>1.43651239789754</v>
+      </c>
+      <c r="AA39">
+        <v>240</v>
+      </c>
+      <c r="AB39">
+        <v>0.77047249571731602</v>
+      </c>
+      <c r="AC39">
+        <v>2000000</v>
+      </c>
+      <c r="AD39">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="40" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y40">
+        <v>4</v>
+      </c>
+      <c r="Z40">
+        <v>1.5291609066156</v>
+      </c>
+      <c r="AA40">
+        <v>240</v>
+      </c>
+      <c r="AB40">
+        <v>0.74402489777622305</v>
+      </c>
+      <c r="AC40">
+        <v>2000000</v>
+      </c>
+      <c r="AD40">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="41" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y41">
+        <v>5</v>
+      </c>
+      <c r="Z41">
+        <v>1.63174028144106</v>
+      </c>
+      <c r="AA41">
+        <v>370</v>
+      </c>
+      <c r="AB41">
+        <v>1.9027261782570299</v>
+      </c>
+      <c r="AC41">
+        <v>2000000</v>
+      </c>
+      <c r="AD41">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="42" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y42">
+        <v>6</v>
+      </c>
+      <c r="Z42">
+        <v>1.73326314317009</v>
+      </c>
+      <c r="AA42">
+        <v>370</v>
+      </c>
+      <c r="AB42">
+        <v>1.9178953936183301</v>
+      </c>
+      <c r="AC42">
+        <v>2000000</v>
+      </c>
+      <c r="AD42">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="43" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y43">
+        <v>7</v>
+      </c>
+      <c r="Z43">
+        <v>1.8344830952098099</v>
+      </c>
+      <c r="AA43">
+        <v>370</v>
+      </c>
+      <c r="AB43">
+        <v>2</v>
+      </c>
+      <c r="AC43">
+        <v>2000000</v>
+      </c>
+      <c r="AD43">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="44" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y44">
+        <v>8</v>
+      </c>
+      <c r="Z44">
+        <v>1.93633394708781</v>
+      </c>
+      <c r="AA44">
+        <v>370</v>
+      </c>
+      <c r="AB44">
+        <v>2</v>
+      </c>
+      <c r="AC44">
+        <v>2000000</v>
+      </c>
+      <c r="AD44">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="45" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y45">
+        <v>9</v>
+      </c>
+      <c r="Z45">
+        <v>2.0452641518224799</v>
+      </c>
+      <c r="AA45">
+        <v>370</v>
+      </c>
+      <c r="AB45">
+        <v>2</v>
+      </c>
+      <c r="AC45">
+        <v>2000000</v>
+      </c>
+      <c r="AD45">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="46" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y46">
+        <v>10</v>
+      </c>
+      <c r="Z46">
+        <v>2.1523191707020302</v>
+      </c>
+      <c r="AA46">
+        <v>370</v>
+      </c>
+      <c r="AB46">
+        <v>2</v>
+      </c>
+      <c r="AC46">
+        <v>2000000</v>
+      </c>
+      <c r="AD46">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="47" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y47">
+        <v>11</v>
+      </c>
+      <c r="Z47">
+        <v>2.2580761461679302</v>
+      </c>
+      <c r="AA47">
+        <v>370</v>
+      </c>
+      <c r="AB47">
+        <v>2</v>
+      </c>
+      <c r="AC47">
+        <v>2000000</v>
+      </c>
+      <c r="AD47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="48" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="Y48">
+        <v>12</v>
+      </c>
+      <c r="Z48">
+        <v>2.3777388265627799</v>
+      </c>
+      <c r="AA48">
+        <v>284</v>
+      </c>
+      <c r="AB48">
+        <v>1.6029833319726401</v>
+      </c>
+      <c r="AC48">
+        <v>2000000</v>
+      </c>
+      <c r="AD48">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="49" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y49">
+        <v>13</v>
+      </c>
+      <c r="Z49">
+        <v>2.49639794926521</v>
+      </c>
+      <c r="AA49">
+        <v>287</v>
+      </c>
+      <c r="AB49">
+        <v>1.65365356228209</v>
+      </c>
+      <c r="AC49">
+        <v>2000000</v>
+      </c>
+      <c r="AD49">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="50" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y50">
+        <v>14</v>
+      </c>
+      <c r="Z50">
+        <v>2.6158093888716598</v>
+      </c>
+      <c r="AA50">
+        <v>290</v>
+      </c>
+      <c r="AB50">
+        <v>1.7259047066175299</v>
+      </c>
+      <c r="AC50">
+        <v>2000000</v>
+      </c>
+      <c r="AD50">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="51" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y51">
+        <v>15</v>
+      </c>
+      <c r="Z51">
+        <v>2.71094462300836</v>
+      </c>
+      <c r="AA51">
+        <v>323</v>
+      </c>
+      <c r="AB51">
+        <v>2</v>
+      </c>
+      <c r="AC51">
+        <v>2000000</v>
+      </c>
+      <c r="AD51">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="52" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y52">
+        <v>16</v>
+      </c>
+      <c r="Z52">
+        <v>2.8522603082045999</v>
+      </c>
+      <c r="AA52">
+        <v>298</v>
+      </c>
+      <c r="AB52">
+        <v>1.81541996575431</v>
+      </c>
+      <c r="AC52">
+        <v>2000000</v>
+      </c>
+      <c r="AD52">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="53" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y53">
+        <v>17</v>
+      </c>
+      <c r="Z53">
+        <v>2.9719790976206601</v>
+      </c>
+      <c r="AA53">
+        <v>295</v>
+      </c>
+      <c r="AB53">
+        <v>1.85732315256537</v>
+      </c>
+      <c r="AC53">
+        <v>2000000</v>
+      </c>
+      <c r="AD53">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="54" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y54">
+        <v>18</v>
+      </c>
+      <c r="Z54">
+        <v>3.0902094245203799</v>
+      </c>
+      <c r="AA54">
+        <v>301</v>
+      </c>
+      <c r="AB54">
+        <v>1.9152752613630399</v>
+      </c>
+      <c r="AC54">
+        <v>2000000</v>
+      </c>
+      <c r="AD54">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="55" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y55">
+        <v>19</v>
+      </c>
+      <c r="Z55">
+        <v>3.2060834969884802</v>
+      </c>
+      <c r="AA55">
+        <v>299</v>
+      </c>
+      <c r="AB55">
+        <v>2</v>
+      </c>
+      <c r="AC55">
+        <v>2000000</v>
+      </c>
+      <c r="AD55">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="56" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y56">
+        <v>20</v>
+      </c>
+      <c r="Z56">
+        <v>3.2979787911071998</v>
+      </c>
+      <c r="AA56">
+        <v>299</v>
+      </c>
+      <c r="AB56">
+        <v>2</v>
+      </c>
+      <c r="AC56">
+        <v>2000000</v>
+      </c>
+      <c r="AD56">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="57" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y57">
+        <v>21</v>
+      </c>
+      <c r="Z57">
+        <v>3.3601181784771201</v>
+      </c>
+      <c r="AA57">
+        <v>295</v>
+      </c>
+      <c r="AB57">
+        <v>2</v>
+      </c>
+      <c r="AC57">
+        <v>2000000</v>
+      </c>
+      <c r="AD57">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="58" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y58">
+        <v>22</v>
+      </c>
+      <c r="Z58">
+        <v>3.4029657145452501</v>
+      </c>
+      <c r="AA58">
+        <v>284</v>
+      </c>
+      <c r="AB58">
+        <v>2</v>
+      </c>
+      <c r="AC58">
+        <v>2000000</v>
+      </c>
+      <c r="AD58">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="59" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y59">
+        <v>23</v>
+      </c>
+      <c r="Z59">
+        <v>3.4253480456309799</v>
+      </c>
+      <c r="AA59">
+        <v>272</v>
+      </c>
+      <c r="AB59">
+        <v>2</v>
+      </c>
+      <c r="AC59">
+        <v>2000000</v>
+      </c>
+      <c r="AD59">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="60" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y60">
+        <v>24</v>
+      </c>
+      <c r="Z60">
+        <v>3.44238874354058</v>
+      </c>
+      <c r="AA60">
+        <v>262</v>
+      </c>
+      <c r="AB60">
+        <v>2</v>
+      </c>
+      <c r="AC60">
+        <v>2000000</v>
+      </c>
+      <c r="AD60">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="61" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y61">
+        <v>25</v>
+      </c>
+      <c r="Z61">
+        <v>3.4657011033449399</v>
+      </c>
+      <c r="AA61">
+        <v>240</v>
+      </c>
+      <c r="AB61">
+        <v>2</v>
+      </c>
+      <c r="AC61">
+        <v>2000000</v>
+      </c>
+      <c r="AD61">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="62" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y62">
+        <v>26</v>
+      </c>
+      <c r="Z62">
+        <v>3.4827335625295399</v>
+      </c>
+      <c r="AA62">
+        <v>240</v>
+      </c>
+      <c r="AB62">
+        <v>2</v>
+      </c>
+      <c r="AC62">
+        <v>2000000</v>
+      </c>
+      <c r="AD62">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="63" spans="25:30" x14ac:dyDescent="0.25">
+      <c r="Y63">
+        <v>27</v>
+      </c>
+      <c r="Z63">
+        <v>3.49976602171414</v>
+      </c>
+      <c r="AA63">
+        <v>240</v>
+      </c>
+      <c r="AB63">
+        <v>2</v>
+      </c>
+      <c r="AC63">
+        <v>2000000</v>
+      </c>
+      <c r="AD63">
+        <v>600</v>
       </c>
     </row>
   </sheetData>
@@ -5096,6 +5915,7 @@
     <mergeCell ref="L2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>